<commit_message>
style: adjust the export format to make it clean and accurate
</commit_message>
<xml_diff>
--- a/procurement_documents/Purchase Order Template.xlsx
+++ b/procurement_documents/Purchase Order Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA93C68-E9C1-4F9E-8663-3696D32D8E97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9058FDA2-B1A1-41FA-9BD6-ED01B45DD3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1AFC0673-2000-41F1-BB87-1A913DCADB25}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="70">
   <si>
     <t>Stock/Property No.</t>
   </si>
@@ -257,6 +257,27 @@
   </si>
   <si>
     <t>*** Nothing follows *** (After the last item)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Place of </t>
+  </si>
+  <si>
+    <t>Delivery:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date of </t>
+  </si>
+  <si>
+    <t xml:space="preserve">REXMELLE </t>
+  </si>
+  <si>
+    <t>F. DECAPIA,</t>
+  </si>
+  <si>
+    <t>JR., Ph.D</t>
+  </si>
+  <si>
+    <t>[po_title]</t>
   </si>
 </sst>
 </file>
@@ -266,7 +287,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +355,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -853,7 +904,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -975,6 +1026,75 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -984,79 +1104,81 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1460,7 +1582,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -1468,82 +1590,82 @@
     <col min="4" max="6" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="e" vm="1">
+    <row r="1" spans="1:8" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="76" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="76"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="78" t="s">
+      <c r="C1" s="68"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="79"/>
-    </row>
-    <row r="2" spans="1:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="74"/>
-      <c r="B2" s="80" t="s">
+      <c r="F1" s="113"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="77"/>
+      <c r="B2" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="82" t="s">
+      <c r="C2" s="72"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="74" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="83"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F2" s="75"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="34"/>
-      <c r="C4" s="84"/>
-      <c r="D4" s="85"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="64"/>
       <c r="E4" s="35" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="54"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="66"/>
       <c r="E5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="55"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66"/>
       <c r="E6" s="40" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="55"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="67"/>
+      <c r="C7" s="78"/>
+      <c r="D7" s="79"/>
       <c r="E7" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="56"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F7" s="107"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>16</v>
       </c>
@@ -1552,43 +1674,48 @@
       <c r="D8" s="29"/>
       <c r="E8" s="29"/>
       <c r="F8" s="30"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H8" s="114"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
-      <c r="B9" s="68" t="s">
+      <c r="B9" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
       <c r="F9" s="15"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="69"/>
-      <c r="D10" s="70"/>
-      <c r="E10" s="41" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="89" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="90" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="80"/>
+      <c r="D10" s="81"/>
+      <c r="E10" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="87"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="42" t="s">
+      <c r="F10" s="61"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="91" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="92" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="82"/>
+      <c r="D11" s="83"/>
+      <c r="E11" s="102" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="88"/>
-    </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="48" t="s">
+      <c r="F11" s="62"/>
+    </row>
+    <row r="12" spans="1:8" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="108" t="s">
         <v>0</v>
       </c>
       <c r="B12" s="49" t="s">
@@ -1607,210 +1734,211 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="59"/>
       <c r="B13" s="1"/>
       <c r="C13" s="6"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="22"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E13" s="103"/>
+      <c r="F13" s="104"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="59"/>
       <c r="B14" s="1"/>
       <c r="C14" s="6"/>
       <c r="D14" s="1"/>
-      <c r="F14" s="22"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E14" s="105"/>
+      <c r="F14" s="104"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="59"/>
       <c r="B15" s="1"/>
       <c r="C15" s="6"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="22"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E15" s="103"/>
+      <c r="F15" s="104"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="59"/>
       <c r="B16" s="1"/>
       <c r="C16" s="6"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="22"/>
+      <c r="E16" s="103"/>
+      <c r="F16" s="104"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="59"/>
       <c r="B17" s="1"/>
       <c r="C17" s="6"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="22"/>
+      <c r="E17" s="103"/>
+      <c r="F17" s="104"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="59"/>
       <c r="B18" s="1"/>
       <c r="C18" s="6"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="22"/>
+      <c r="E18" s="103"/>
+      <c r="F18" s="104"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="59"/>
       <c r="B19" s="1"/>
       <c r="C19" s="6"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="22"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="104"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="59"/>
       <c r="B20" s="1"/>
       <c r="C20" s="6"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="22"/>
+      <c r="E20" s="103"/>
+      <c r="F20" s="104"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="59"/>
       <c r="B21" s="1"/>
       <c r="C21" s="6"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="22"/>
+      <c r="E21" s="103"/>
+      <c r="F21" s="104"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="59"/>
       <c r="B22" s="1"/>
       <c r="C22" s="6"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="22"/>
+      <c r="E22" s="103"/>
+      <c r="F22" s="104"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="59"/>
       <c r="B23" s="1"/>
       <c r="C23" s="6"/>
       <c r="D23" s="1"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="22"/>
+      <c r="E23" s="103"/>
+      <c r="F23" s="104"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="59"/>
       <c r="B24" s="1"/>
       <c r="C24" s="6"/>
       <c r="D24" s="1"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="22"/>
+      <c r="E24" s="103"/>
+      <c r="F24" s="104"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="59"/>
       <c r="B25" s="1"/>
       <c r="C25" s="6"/>
       <c r="D25" s="1"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="22"/>
+      <c r="E25" s="103"/>
+      <c r="F25" s="104"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="59"/>
       <c r="B26" s="1"/>
       <c r="C26" s="6"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="22"/>
+      <c r="E26" s="103"/>
+      <c r="F26" s="104"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="59"/>
       <c r="B27" s="1"/>
       <c r="C27" s="6"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="22"/>
+      <c r="E27" s="103"/>
+      <c r="F27" s="104"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="59"/>
       <c r="B28" s="1"/>
       <c r="C28" s="6"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="22"/>
+      <c r="E28" s="103"/>
+      <c r="F28" s="104"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
       <c r="B29" s="1"/>
       <c r="C29" s="6"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="22"/>
+      <c r="E29" s="103"/>
+      <c r="F29" s="104"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="59"/>
       <c r="B30" s="1"/>
       <c r="C30" s="6"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="22"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="104"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="59"/>
       <c r="B31" s="1"/>
       <c r="C31" s="6"/>
       <c r="D31" s="1"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="22"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="104"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
       <c r="B32" s="1"/>
       <c r="C32" s="6"/>
       <c r="D32" s="1"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="22"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="104"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
       <c r="B33" s="1"/>
       <c r="C33" s="6"/>
       <c r="D33" s="1"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="22"/>
+      <c r="E33" s="103"/>
+      <c r="F33" s="104"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="59"/>
       <c r="B34" s="1"/>
       <c r="C34" s="6"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="22"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="104"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="59"/>
       <c r="B35" s="1"/>
       <c r="C35" s="6"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="22"/>
+      <c r="E35" s="103"/>
+      <c r="F35" s="104"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="59"/>
       <c r="B36" s="1"/>
       <c r="C36" s="6"/>
       <c r="D36" s="1"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="22"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="104"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="59"/>
       <c r="B37" s="1"/>
       <c r="C37" s="6"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="22"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="104"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="23"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="47" t="s">
-        <v>6</v>
+      <c r="C38" s="110" t="s">
+        <v>69</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -1819,79 +1947,106 @@
     <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="25"/>
       <c r="B39" s="26"/>
-      <c r="C39" s="27" t="s">
+      <c r="C39" s="111" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="26"/>
       <c r="E39" s="26"/>
-      <c r="F39" s="36" t="s">
+      <c r="F39" s="106" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="61" t="s">
+      <c r="A41" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="62"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="62"/>
-      <c r="E41" s="62"/>
-      <c r="F41" s="63"/>
+      <c r="B41" s="85"/>
+      <c r="C41" s="85"/>
+      <c r="D41" s="85"/>
+      <c r="E41" s="85"/>
+      <c r="F41" s="86"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12"/>
+      <c r="B42" s="93"/>
+      <c r="C42" s="93"/>
+      <c r="D42" s="93"/>
+      <c r="E42" s="93"/>
       <c r="F42" s="13"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12"/>
-      <c r="B43" s="53" t="s">
+      <c r="B43" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="C43" s="93"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="109" t="s">
         <v>26</v>
       </c>
       <c r="F43" s="13"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12"/>
-      <c r="E44" s="86" t="s">
-        <v>27</v>
-      </c>
-      <c r="F44" s="13"/>
+      <c r="B44" s="93"/>
+      <c r="C44" s="93"/>
+      <c r="D44" s="95" t="s">
+        <v>66</v>
+      </c>
+      <c r="E44" s="96" t="s">
+        <v>67</v>
+      </c>
+      <c r="F44" s="97" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="12"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
-      <c r="E45" s="3" t="s">
+      <c r="D45" s="93"/>
+      <c r="E45" s="109" t="s">
         <v>28</v>
       </c>
       <c r="F45" s="13"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12"/>
-      <c r="C46" s="44" t="s">
+      <c r="B46" s="93"/>
+      <c r="C46" s="98" t="s">
         <v>30</v>
       </c>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
       <c r="F46" s="13"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12"/>
+      <c r="B47" s="93"/>
+      <c r="C47" s="93"/>
+      <c r="D47" s="93"/>
+      <c r="E47" s="93"/>
       <c r="F47" s="13"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12"/>
-      <c r="C48" s="44" t="s">
+      <c r="B48" s="93"/>
+      <c r="C48" s="98" t="s">
         <v>31</v>
       </c>
+      <c r="D48" s="93"/>
+      <c r="E48" s="93"/>
       <c r="F48" s="13"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="12"/>
-      <c r="C49" s="45" t="s">
+      <c r="B49" s="93"/>
+      <c r="C49" s="99" t="s">
         <v>43</v>
       </c>
+      <c r="D49" s="93"/>
+      <c r="E49" s="93"/>
       <c r="F49" s="13"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -1911,7 +2066,7 @@
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="8"/>
-      <c r="E51" s="43" t="s">
+      <c r="E51" s="88" t="s">
         <v>37</v>
       </c>
       <c r="F51" s="16" t="s">
@@ -1919,12 +2074,13 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="38" t="s">
+      <c r="A52" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="93" t="s">
         <v>34</v>
       </c>
+      <c r="C52" s="93"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10" t="s">
         <v>38</v>
@@ -1935,6 +2091,8 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="12"/>
+      <c r="B53" s="93"/>
+      <c r="C53" s="93"/>
       <c r="D53" s="11"/>
       <c r="E53" s="10" t="s">
         <v>39</v>
@@ -1945,7 +2103,8 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="12"/>
-      <c r="C54" s="51" t="s">
+      <c r="B54" s="93"/>
+      <c r="C54" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D54" s="11"/>
@@ -1964,23 +2123,23 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="B9:E9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="92" fitToWidth="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="93" fitToWidth="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1998,30 +2157,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="e" vm="1">
+      <c r="A1" s="76" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="76"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="78" t="s">
+      <c r="C1" s="68"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="79"/>
+      <c r="F1" s="71"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="74"/>
-      <c r="B2" s="80" t="s">
+      <c r="A2" s="77"/>
+      <c r="B2" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="82" t="s">
+      <c r="C2" s="72"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="74" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="83"/>
+      <c r="F2" s="75"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2029,10 +2188,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="34"/>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="85"/>
+      <c r="D4" s="64"/>
       <c r="E4" s="35" t="s">
         <v>20</v>
       </c>
@@ -2045,10 +2204,10 @@
         <v>13</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="64" t="s">
+      <c r="C5" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="65"/>
+      <c r="D5" s="66"/>
       <c r="E5" s="5" t="s">
         <v>21</v>
       </c>
@@ -2061,10 +2220,10 @@
         <v>14</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="65"/>
+      <c r="D6" s="66"/>
       <c r="E6" s="40" t="s">
         <v>22</v>
       </c>
@@ -2077,10 +2236,10 @@
         <v>15</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="C7" s="66" t="s">
+      <c r="C7" s="78" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="67"/>
+      <c r="D7" s="79"/>
       <c r="E7" s="39" t="s">
         <v>23</v>
       </c>
@@ -2100,12 +2259,12 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
-      <c r="B9" s="68" t="s">
+      <c r="B9" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
       <c r="F9" s="15"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2113,10 +2272,10 @@
         <v>18</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="C10" s="69" t="s">
+      <c r="C10" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="70"/>
+      <c r="D10" s="81"/>
       <c r="E10" s="41" t="s">
         <v>24</v>
       </c>
@@ -2129,10 +2288,10 @@
         <v>19</v>
       </c>
       <c r="B11" s="32"/>
-      <c r="C11" s="71" t="s">
+      <c r="C11" s="82" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="72"/>
+      <c r="D11" s="83"/>
       <c r="E11" s="42" t="s">
         <v>25</v>
       </c>
@@ -2397,14 +2556,14 @@
     </row>
     <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="61" t="s">
+      <c r="A41" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="62"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="62"/>
-      <c r="E41" s="62"/>
-      <c r="F41" s="63"/>
+      <c r="B41" s="85"/>
+      <c r="C41" s="85"/>
+      <c r="D41" s="85"/>
+      <c r="E41" s="85"/>
+      <c r="F41" s="86"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12"/>
@@ -2531,12 +2690,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:F2"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
@@ -2544,6 +2697,12 @@
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:F2"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>